<commit_message>
Remove master_dataset_summary.txt, now redundant with the README
The file described the master table - participant count, row count, rows per
phase and the column list - all of which the rewritten README section now
carries. Its one unique claim, that no participant is missing an extracted
file, pain data or anthropometrics, is folded into the README instead.
</commit_message>
<xml_diff>
--- a/data/files_help/combined_data_boolian_vas.xlsx
+++ b/data/files_help/combined_data_boolian_vas.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/688a6d66afb8592b/שולחן העבודה/neck_in_cycling/Results/files_help/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/omerpeled/ph.d_repo/data/files_help/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="18" documentId="11_BDEBB499094492908BE4B30C05F58D3174DA8CA7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0224AA14-672F-7B42-A8F1-151E806F904C}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8336A5F9-D3E6-E94E-918C-FD5D76E156E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15900" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,9 +44,6 @@
     <t>cluster</t>
   </si>
   <si>
-    <t>pain_bulian</t>
-  </si>
-  <si>
     <t>vas</t>
   </si>
   <si>
@@ -228,6 +225,9 @@
   </si>
   <si>
     <t>632</t>
+  </si>
+  <si>
+    <t>pain_boolian</t>
   </si>
 </sst>
 </file>
@@ -518,18 +518,18 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>3</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -543,7 +543,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -557,7 +557,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -571,7 +571,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -585,7 +585,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -599,7 +599,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B7">
         <v>1</v>
@@ -613,7 +613,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B8">
         <v>1</v>
@@ -627,7 +627,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B9">
         <v>0</v>
@@ -652,7 +652,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B11">
         <v>0</v>
@@ -666,7 +666,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B12">
         <v>0</v>
@@ -680,7 +680,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B13">
         <v>1</v>
@@ -694,7 +694,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B14">
         <v>1</v>
@@ -708,7 +708,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B15">
         <v>0</v>
@@ -722,7 +722,7 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B16">
         <v>0</v>
@@ -736,7 +736,7 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B17">
         <v>0</v>
@@ -750,7 +750,7 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B18">
         <v>0</v>
@@ -764,7 +764,7 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B19">
         <v>1</v>
@@ -778,7 +778,7 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B20">
         <v>0</v>
@@ -792,7 +792,7 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B21">
         <v>0</v>
@@ -806,7 +806,7 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B22">
         <v>0</v>
@@ -820,7 +820,7 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B23">
         <v>0</v>
@@ -834,7 +834,7 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B24">
         <v>0</v>
@@ -848,7 +848,7 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B25">
         <v>1</v>
@@ -862,7 +862,7 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B26">
         <v>0</v>
@@ -876,7 +876,7 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B27">
         <v>0</v>
@@ -904,7 +904,7 @@
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B29">
         <v>0</v>
@@ -918,7 +918,7 @@
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B30">
         <v>0</v>
@@ -932,7 +932,7 @@
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B31">
         <v>1</v>
@@ -946,7 +946,7 @@
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B32">
         <v>0</v>
@@ -960,7 +960,7 @@
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B33">
         <v>0</v>
@@ -974,7 +974,7 @@
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B34">
         <v>1</v>
@@ -988,7 +988,7 @@
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B35">
         <v>0</v>
@@ -1002,7 +1002,7 @@
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B36">
         <v>0</v>
@@ -1016,7 +1016,7 @@
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B37">
         <v>0</v>
@@ -1030,7 +1030,7 @@
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B38">
         <v>0</v>
@@ -1044,7 +1044,7 @@
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B39">
         <v>0</v>
@@ -1058,7 +1058,7 @@
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B40">
         <v>0</v>
@@ -1072,7 +1072,7 @@
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B41">
         <v>0</v>
@@ -1086,7 +1086,7 @@
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B42">
         <v>0</v>
@@ -1100,7 +1100,7 @@
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B43">
         <v>0</v>
@@ -1114,7 +1114,7 @@
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B44">
         <v>1</v>
@@ -1128,7 +1128,7 @@
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B45">
         <v>0</v>
@@ -1142,7 +1142,7 @@
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B46">
         <v>1</v>
@@ -1156,7 +1156,7 @@
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B47">
         <v>0</v>
@@ -1170,7 +1170,7 @@
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B48">
         <v>0</v>
@@ -1184,7 +1184,7 @@
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B49">
         <v>1</v>
@@ -1198,7 +1198,7 @@
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B50">
         <v>0</v>
@@ -1212,7 +1212,7 @@
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B51">
         <v>0</v>
@@ -1226,7 +1226,7 @@
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B52">
         <v>0</v>
@@ -1240,7 +1240,7 @@
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B53">
         <v>1</v>
@@ -1254,7 +1254,7 @@
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B54">
         <v>0</v>
@@ -1268,7 +1268,7 @@
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B55">
         <v>0</v>
@@ -1282,7 +1282,7 @@
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B56">
         <v>0</v>
@@ -1296,7 +1296,7 @@
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B57">
         <v>1</v>
@@ -1310,7 +1310,7 @@
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B58">
         <v>0</v>
@@ -1324,7 +1324,7 @@
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B59">
         <v>0</v>
@@ -1338,7 +1338,7 @@
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B60">
         <v>0</v>
@@ -1352,7 +1352,7 @@
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B61">
         <v>1</v>
@@ -1366,7 +1366,7 @@
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B62">
         <v>0</v>

</xml_diff>